<commit_message>
Correction in count of articles per database
</commit_message>
<xml_diff>
--- a/survey_info.xlsx
+++ b/survey_info.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sofiamorgado/Desktop/phd_sofia/survey/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sofiamorgado/Desktop/survey_ml_cad/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21555D4A-7A99-8444-ABE0-80DA3782EBCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CB24918-80A6-7F4B-9671-3515E2D5F7AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="880" yWindow="780" windowWidth="32800" windowHeight="19780" activeTab="1" xr2:uid="{775E742D-3574-834D-BFD8-73EB03BF95DA}"/>
+    <workbookView xWindow="-500" yWindow="780" windowWidth="19820" windowHeight="19780" xr2:uid="{775E742D-3574-834D-BFD8-73EB03BF95DA}"/>
   </bookViews>
   <sheets>
     <sheet name="search_queries" sheetId="2" r:id="rId1"/>
@@ -4781,7 +4781,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="14">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -5404,7 +5404,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88A7BFA9-7709-4346-9D75-A3427D7883F1}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="20.6640625" customWidth="1"/>
     <col min="2" max="2" width="95.1640625" customWidth="1"/>
@@ -5412,7 +5412,7 @@
     <col min="4" max="4" width="19.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -5426,7 +5426,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" ht="60" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -5440,7 +5440,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" ht="60" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -5451,10 +5451,10 @@
         <v>84</v>
       </c>
       <c r="D3" s="18">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="60" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -5465,10 +5465,10 @@
         <v>86</v>
       </c>
       <c r="D4" s="18">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="60" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
@@ -5482,7 +5482,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" ht="20" customHeight="1">
       <c r="A6" s="5" t="s">
         <v>22</v>
       </c>
@@ -5505,7 +5505,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E900737-FDAA-0044-A9B4-DF588C19E6A2}">
   <dimension ref="A1:AE346"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="4" width="19.33203125" customWidth="1"/>
     <col min="5" max="5" width="17.5" customWidth="1"/>
@@ -5521,7 +5521,7 @@
     <col min="31" max="31" width="83.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:31" ht="17">
       <c r="A1" s="6" t="s">
         <v>4</v>
       </c>
@@ -5616,7 +5616,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:31" ht="17">
       <c r="A2" s="4" t="s">
         <v>6</v>
       </c>
@@ -5657,7 +5657,7 @@
       <c r="AD2" s="8"/>
       <c r="AE2" s="8"/>
     </row>
-    <row r="3" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:31" ht="17">
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
@@ -5698,7 +5698,7 @@
       <c r="AD3" s="8"/>
       <c r="AE3" s="8"/>
     </row>
-    <row r="4" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:31" ht="17">
       <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
@@ -5739,7 +5739,7 @@
       <c r="AD4" s="8"/>
       <c r="AE4" s="8"/>
     </row>
-    <row r="5" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:31" ht="17">
       <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
@@ -5780,7 +5780,7 @@
       <c r="AD5" s="8"/>
       <c r="AE5" s="8"/>
     </row>
-    <row r="6" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:31" ht="17">
       <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
@@ -5821,7 +5821,7 @@
       <c r="AD6" s="8"/>
       <c r="AE6" s="8"/>
     </row>
-    <row r="7" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:31" ht="17">
       <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
@@ -5862,7 +5862,7 @@
       <c r="AD7" s="8"/>
       <c r="AE7" s="8"/>
     </row>
-    <row r="8" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:31" ht="17">
       <c r="A8" s="4" t="s">
         <v>6</v>
       </c>
@@ -5903,7 +5903,7 @@
       <c r="AD8" s="8"/>
       <c r="AE8" s="8"/>
     </row>
-    <row r="9" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:31" ht="17">
       <c r="A9" s="4" t="s">
         <v>6</v>
       </c>
@@ -5944,7 +5944,7 @@
       <c r="AD9" s="8"/>
       <c r="AE9" s="8"/>
     </row>
-    <row r="10" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:31" ht="17">
       <c r="A10" s="4" t="s">
         <v>6</v>
       </c>
@@ -5985,7 +5985,7 @@
       <c r="AD10" s="8"/>
       <c r="AE10" s="8"/>
     </row>
-    <row r="11" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:31" ht="17">
       <c r="A11" s="4" t="s">
         <v>6</v>
       </c>
@@ -6026,7 +6026,7 @@
       <c r="AD11" s="8"/>
       <c r="AE11" s="8"/>
     </row>
-    <row r="12" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:31" ht="17">
       <c r="A12" s="4" t="s">
         <v>6</v>
       </c>
@@ -6067,7 +6067,7 @@
       <c r="AD12" s="8"/>
       <c r="AE12" s="8"/>
     </row>
-    <row r="13" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:31" ht="17">
       <c r="A13" s="4" t="s">
         <v>6</v>
       </c>
@@ -6108,7 +6108,7 @@
       <c r="AD13" s="8"/>
       <c r="AE13" s="8"/>
     </row>
-    <row r="14" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:31" ht="17">
       <c r="A14" s="4" t="s">
         <v>6</v>
       </c>
@@ -6149,7 +6149,7 @@
       <c r="AD14" s="8"/>
       <c r="AE14" s="8"/>
     </row>
-    <row r="15" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:31" ht="17">
       <c r="A15" s="4" t="s">
         <v>6</v>
       </c>
@@ -6190,7 +6190,7 @@
       <c r="AD15" s="8"/>
       <c r="AE15" s="8"/>
     </row>
-    <row r="16" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:31" ht="17">
       <c r="A16" s="4" t="s">
         <v>6</v>
       </c>
@@ -6231,7 +6231,7 @@
       <c r="AD16" s="8"/>
       <c r="AE16" s="8"/>
     </row>
-    <row r="17" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:31" ht="17">
       <c r="A17" s="4" t="s">
         <v>6</v>
       </c>
@@ -6272,7 +6272,7 @@
       <c r="AD17" s="8"/>
       <c r="AE17" s="8"/>
     </row>
-    <row r="18" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:31" ht="17">
       <c r="A18" s="4" t="s">
         <v>6</v>
       </c>
@@ -6313,7 +6313,7 @@
       <c r="AD18" s="8"/>
       <c r="AE18" s="8"/>
     </row>
-    <row r="19" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:31" ht="17">
       <c r="A19" s="4" t="s">
         <v>6</v>
       </c>
@@ -6354,7 +6354,7 @@
       <c r="AD19" s="8"/>
       <c r="AE19" s="8"/>
     </row>
-    <row r="20" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:31" ht="255">
       <c r="A20" s="4" t="s">
         <v>6</v>
       </c>
@@ -6447,7 +6447,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="21" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:31" ht="17">
       <c r="A21" s="4" t="s">
         <v>6</v>
       </c>
@@ -6488,7 +6488,7 @@
       <c r="AD21" s="16"/>
       <c r="AE21" s="17"/>
     </row>
-    <row r="22" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:31" ht="17">
       <c r="A22" s="4" t="s">
         <v>6</v>
       </c>
@@ -6529,7 +6529,7 @@
       <c r="AD22" s="8"/>
       <c r="AE22" s="8"/>
     </row>
-    <row r="23" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:31" ht="255">
       <c r="A23" s="4" t="s">
         <v>6</v>
       </c>
@@ -6620,7 +6620,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="24" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:31" ht="17">
       <c r="A24" s="4" t="s">
         <v>6</v>
       </c>
@@ -6661,7 +6661,7 @@
       <c r="AD24" s="8"/>
       <c r="AE24" s="8"/>
     </row>
-    <row r="25" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:31" ht="17">
       <c r="A25" s="4" t="s">
         <v>6</v>
       </c>
@@ -6702,7 +6702,7 @@
       <c r="AD25" s="8"/>
       <c r="AE25" s="8"/>
     </row>
-    <row r="26" spans="1:31" ht="221" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:31" ht="221">
       <c r="A26" s="4" t="s">
         <v>6</v>
       </c>
@@ -6795,7 +6795,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="27" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:31" ht="17">
       <c r="A27" s="4" t="s">
         <v>6</v>
       </c>
@@ -6836,7 +6836,7 @@
       <c r="AD27" s="8"/>
       <c r="AE27" s="8"/>
     </row>
-    <row r="28" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:31" ht="17">
       <c r="A28" s="4" t="s">
         <v>6</v>
       </c>
@@ -6877,7 +6877,7 @@
       <c r="AD28" s="8"/>
       <c r="AE28" s="8"/>
     </row>
-    <row r="29" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:31" ht="17">
       <c r="A29" s="4" t="s">
         <v>6</v>
       </c>
@@ -6918,7 +6918,7 @@
       <c r="AD29" s="8"/>
       <c r="AE29" s="8"/>
     </row>
-    <row r="30" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:31" ht="17">
       <c r="A30" s="4" t="s">
         <v>6</v>
       </c>
@@ -6959,7 +6959,7 @@
       <c r="AD30" s="8"/>
       <c r="AE30" s="8"/>
     </row>
-    <row r="31" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:31" ht="17">
       <c r="A31" s="4" t="s">
         <v>6</v>
       </c>
@@ -7000,7 +7000,7 @@
       <c r="AD31" s="8"/>
       <c r="AE31" s="8"/>
     </row>
-    <row r="32" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:31" ht="17">
       <c r="A32" s="4" t="s">
         <v>6</v>
       </c>
@@ -7041,7 +7041,7 @@
       <c r="AD32" s="8"/>
       <c r="AE32" s="8"/>
     </row>
-    <row r="33" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:31" ht="17">
       <c r="A33" s="4" t="s">
         <v>6</v>
       </c>
@@ -7082,7 +7082,7 @@
       <c r="AD33" s="8"/>
       <c r="AE33" s="8"/>
     </row>
-    <row r="34" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:31" ht="17">
       <c r="A34" s="4" t="s">
         <v>6</v>
       </c>
@@ -7123,7 +7123,7 @@
       <c r="AD34" s="8"/>
       <c r="AE34" s="8"/>
     </row>
-    <row r="35" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:31" ht="17">
       <c r="A35" s="4" t="s">
         <v>6</v>
       </c>
@@ -7164,7 +7164,7 @@
       <c r="AD35" s="8"/>
       <c r="AE35" s="8"/>
     </row>
-    <row r="36" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:31" ht="17">
       <c r="A36" s="4" t="s">
         <v>6</v>
       </c>
@@ -7205,7 +7205,7 @@
       <c r="AD36" s="8"/>
       <c r="AE36" s="8"/>
     </row>
-    <row r="37" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:31" ht="17">
       <c r="A37" s="4" t="s">
         <v>6</v>
       </c>
@@ -7246,7 +7246,7 @@
       <c r="AD37" s="8"/>
       <c r="AE37" s="8"/>
     </row>
-    <row r="38" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:31" ht="17">
       <c r="A38" s="4" t="s">
         <v>6</v>
       </c>
@@ -7287,7 +7287,7 @@
       <c r="AD38" s="8"/>
       <c r="AE38" s="8"/>
     </row>
-    <row r="39" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:31" ht="17">
       <c r="A39" s="4" t="s">
         <v>6</v>
       </c>
@@ -7328,7 +7328,7 @@
       <c r="AD39" s="8"/>
       <c r="AE39" s="8"/>
     </row>
-    <row r="40" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:31" ht="17">
       <c r="A40" s="4" t="s">
         <v>6</v>
       </c>
@@ -7369,7 +7369,7 @@
       <c r="AD40" s="8"/>
       <c r="AE40" s="8"/>
     </row>
-    <row r="41" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:31" ht="17">
       <c r="A41" s="4" t="s">
         <v>6</v>
       </c>
@@ -7410,7 +7410,7 @@
       <c r="AD41" s="8"/>
       <c r="AE41" s="8"/>
     </row>
-    <row r="42" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:31" ht="17">
       <c r="A42" s="4" t="s">
         <v>6</v>
       </c>
@@ -7451,7 +7451,7 @@
       <c r="AD42" s="8"/>
       <c r="AE42" s="8"/>
     </row>
-    <row r="43" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:31" ht="17">
       <c r="A43" s="4" t="s">
         <v>6</v>
       </c>
@@ -7492,7 +7492,7 @@
       <c r="AD43" s="8"/>
       <c r="AE43" s="8"/>
     </row>
-    <row r="44" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:31" ht="17">
       <c r="A44" s="4" t="s">
         <v>6</v>
       </c>
@@ -7533,7 +7533,7 @@
       <c r="AD44" s="8"/>
       <c r="AE44" s="8"/>
     </row>
-    <row r="45" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:31" ht="17">
       <c r="A45" s="4" t="s">
         <v>6</v>
       </c>
@@ -7574,7 +7574,7 @@
       <c r="AD45" s="8"/>
       <c r="AE45" s="8"/>
     </row>
-    <row r="46" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:31" ht="17">
       <c r="A46" s="4" t="s">
         <v>6</v>
       </c>
@@ -7615,7 +7615,7 @@
       <c r="AD46" s="8"/>
       <c r="AE46" s="8"/>
     </row>
-    <row r="47" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:31" ht="17">
       <c r="A47" s="4" t="s">
         <v>6</v>
       </c>
@@ -7656,7 +7656,7 @@
       <c r="AD47" s="8"/>
       <c r="AE47" s="8"/>
     </row>
-    <row r="48" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:31" ht="289">
       <c r="A48" s="4" t="s">
         <v>7</v>
       </c>
@@ -7745,7 +7745,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="49" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:31" ht="255">
       <c r="A49" s="4" t="s">
         <v>7</v>
       </c>
@@ -7838,7 +7838,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="50" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:31" ht="289">
       <c r="A50" s="4" t="s">
         <v>7</v>
       </c>
@@ -7929,7 +7929,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="51" spans="1:31" ht="340" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:31" ht="340">
       <c r="A51" s="4" t="s">
         <v>7</v>
       </c>
@@ -8022,7 +8022,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="52" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:31" ht="289">
       <c r="A52" s="4" t="s">
         <v>7</v>
       </c>
@@ -8113,7 +8113,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="53" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:31" ht="17">
       <c r="A53" s="4" t="s">
         <v>7</v>
       </c>
@@ -8154,7 +8154,7 @@
       <c r="AD53" s="8"/>
       <c r="AE53" s="8"/>
     </row>
-    <row r="54" spans="1:31" ht="323" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:31" ht="323">
       <c r="A54" s="4" t="s">
         <v>7</v>
       </c>
@@ -8245,7 +8245,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="55" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:31" ht="17">
       <c r="A55" s="4" t="s">
         <v>7</v>
       </c>
@@ -8286,7 +8286,7 @@
       <c r="AD55" s="8"/>
       <c r="AE55" s="8"/>
     </row>
-    <row r="56" spans="1:31" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:31" ht="409.6">
       <c r="A56" s="4" t="s">
         <v>10</v>
       </c>
@@ -8377,7 +8377,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="57" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:31" ht="17">
       <c r="A57" s="4" t="s">
         <v>7</v>
       </c>
@@ -8418,7 +8418,7 @@
       <c r="AD57" s="8"/>
       <c r="AE57" s="8"/>
     </row>
-    <row r="58" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:31" ht="17">
       <c r="A58" s="4" t="s">
         <v>7</v>
       </c>
@@ -8459,7 +8459,7 @@
       <c r="AD58" s="8"/>
       <c r="AE58" s="8"/>
     </row>
-    <row r="59" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:31" ht="17">
       <c r="A59" s="4" t="s">
         <v>7</v>
       </c>
@@ -8500,7 +8500,7 @@
       <c r="AD59" s="8"/>
       <c r="AE59" s="8"/>
     </row>
-    <row r="60" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:31" ht="17">
       <c r="A60" s="4" t="s">
         <v>7</v>
       </c>
@@ -8541,7 +8541,7 @@
       <c r="AD60" s="8"/>
       <c r="AE60" s="8"/>
     </row>
-    <row r="61" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:31" ht="17">
       <c r="A61" s="4" t="s">
         <v>10</v>
       </c>
@@ -8582,7 +8582,7 @@
       <c r="AD61" s="8"/>
       <c r="AE61" s="8"/>
     </row>
-    <row r="62" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:31" ht="17">
       <c r="A62" s="4" t="s">
         <v>7</v>
       </c>
@@ -8623,7 +8623,7 @@
       <c r="AD62" s="8"/>
       <c r="AE62" s="8"/>
     </row>
-    <row r="63" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:31" ht="17">
       <c r="A63" s="4" t="s">
         <v>7</v>
       </c>
@@ -8664,7 +8664,7 @@
       <c r="AD63" s="8"/>
       <c r="AE63" s="8"/>
     </row>
-    <row r="64" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:31" ht="272">
       <c r="A64" s="4" t="s">
         <v>10</v>
       </c>
@@ -8755,7 +8755,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="65" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:31" ht="17">
       <c r="A65" s="4" t="s">
         <v>7</v>
       </c>
@@ -8796,7 +8796,7 @@
       <c r="AD65" s="8"/>
       <c r="AE65" s="8"/>
     </row>
-    <row r="66" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:31" ht="17">
       <c r="A66" s="4" t="s">
         <v>7</v>
       </c>
@@ -8837,7 +8837,7 @@
       <c r="AD66" s="16"/>
       <c r="AE66" s="17"/>
     </row>
-    <row r="67" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:31" ht="17">
       <c r="A67" s="4" t="s">
         <v>7</v>
       </c>
@@ -8878,7 +8878,7 @@
       <c r="AD67" s="16"/>
       <c r="AE67" s="17"/>
     </row>
-    <row r="68" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:31" ht="17">
       <c r="A68" s="4" t="s">
         <v>7</v>
       </c>
@@ -8919,7 +8919,7 @@
       <c r="AD68" s="8"/>
       <c r="AE68" s="8"/>
     </row>
-    <row r="69" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:31" ht="17">
       <c r="A69" s="4" t="s">
         <v>7</v>
       </c>
@@ -8960,7 +8960,7 @@
       <c r="AD69" s="8"/>
       <c r="AE69" s="8"/>
     </row>
-    <row r="70" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:31" ht="255">
       <c r="A70" s="4" t="s">
         <v>7</v>
       </c>
@@ -9051,7 +9051,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="71" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:31" ht="255">
       <c r="A71" s="4" t="s">
         <v>7</v>
       </c>
@@ -9144,7 +9144,7 @@
         <v>1018</v>
       </c>
     </row>
-    <row r="72" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:31" ht="17">
       <c r="A72" s="4" t="s">
         <v>7</v>
       </c>
@@ -9185,7 +9185,7 @@
       <c r="AD72" s="8"/>
       <c r="AE72" s="8"/>
     </row>
-    <row r="73" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:31" ht="17">
       <c r="A73" s="4" t="s">
         <v>7</v>
       </c>
@@ -9226,7 +9226,7 @@
       <c r="AD73" s="8"/>
       <c r="AE73" s="8"/>
     </row>
-    <row r="74" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:31" ht="17">
       <c r="A74" s="4" t="s">
         <v>7</v>
       </c>
@@ -9267,7 +9267,7 @@
       <c r="AD74" s="8"/>
       <c r="AE74" s="8"/>
     </row>
-    <row r="75" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:31" ht="17">
       <c r="A75" s="4" t="s">
         <v>7</v>
       </c>
@@ -9308,7 +9308,7 @@
       <c r="AD75" s="8"/>
       <c r="AE75" s="8"/>
     </row>
-    <row r="76" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:31" ht="17">
       <c r="A76" s="4" t="s">
         <v>7</v>
       </c>
@@ -9347,7 +9347,7 @@
       <c r="AD76" s="8"/>
       <c r="AE76" s="8"/>
     </row>
-    <row r="77" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:31" ht="289">
       <c r="A77" s="4" t="s">
         <v>7</v>
       </c>
@@ -9438,7 +9438,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="78" spans="1:31" ht="51" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:31" ht="51">
       <c r="A78" s="4" t="s">
         <v>7</v>
       </c>
@@ -9483,7 +9483,7 @@
       </c>
       <c r="AE78" s="8"/>
     </row>
-    <row r="79" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:31" ht="17">
       <c r="A79" s="4" t="s">
         <v>7</v>
       </c>
@@ -9524,7 +9524,7 @@
       <c r="AD79" s="8"/>
       <c r="AE79" s="8"/>
     </row>
-    <row r="80" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:31" ht="17">
       <c r="A80" s="4" t="s">
         <v>10</v>
       </c>
@@ -9565,7 +9565,7 @@
       <c r="AD80" s="8"/>
       <c r="AE80" s="8"/>
     </row>
-    <row r="81" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:31" ht="272">
       <c r="A81" s="4" t="s">
         <v>10</v>
       </c>
@@ -9656,7 +9656,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="82" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:31" ht="17">
       <c r="A82" s="4" t="s">
         <v>7</v>
       </c>
@@ -9697,7 +9697,7 @@
       <c r="AD82" s="8"/>
       <c r="AE82" s="8"/>
     </row>
-    <row r="83" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:31" ht="272">
       <c r="A83" s="4" t="s">
         <v>10</v>
       </c>
@@ -9790,7 +9790,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="84" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:31" ht="255">
       <c r="A84" s="4" t="s">
         <v>7</v>
       </c>
@@ -9883,7 +9883,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="85" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:31" ht="17">
       <c r="A85" s="4" t="s">
         <v>7</v>
       </c>
@@ -9926,7 +9926,7 @@
       <c r="AD85" s="8"/>
       <c r="AE85" s="8"/>
     </row>
-    <row r="86" spans="1:31" ht="306" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:31" ht="306">
       <c r="A86" s="4" t="s">
         <v>10</v>
       </c>
@@ -10017,7 +10017,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="87" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:31" ht="17">
       <c r="A87" s="4" t="s">
         <v>7</v>
       </c>
@@ -10058,7 +10058,7 @@
       <c r="AD87" s="8"/>
       <c r="AE87" s="8"/>
     </row>
-    <row r="88" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:31" ht="255">
       <c r="A88" s="4" t="s">
         <v>7</v>
       </c>
@@ -10149,7 +10149,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="89" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:31" ht="289">
       <c r="A89" s="4" t="s">
         <v>7</v>
       </c>
@@ -10240,7 +10240,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="90" spans="1:31" ht="238" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:31" ht="238">
       <c r="A90" s="4" t="s">
         <v>7</v>
       </c>
@@ -10331,7 +10331,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="91" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:31" ht="17">
       <c r="A91" s="4" t="s">
         <v>7</v>
       </c>
@@ -10372,7 +10372,7 @@
       <c r="AD91" s="8"/>
       <c r="AE91" s="8"/>
     </row>
-    <row r="92" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:31" ht="17">
       <c r="A92" s="4" t="s">
         <v>7</v>
       </c>
@@ -10413,7 +10413,7 @@
       <c r="AD92" s="8"/>
       <c r="AE92" s="8"/>
     </row>
-    <row r="93" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:31" ht="272">
       <c r="A93" s="4" t="s">
         <v>7</v>
       </c>
@@ -10506,7 +10506,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="94" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:31" ht="255">
       <c r="A94" s="4" t="s">
         <v>7</v>
       </c>
@@ -10597,7 +10597,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="95" spans="1:31" ht="238" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:31" ht="238">
       <c r="A95" s="4" t="s">
         <v>10</v>
       </c>
@@ -10688,7 +10688,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="96" spans="1:31" ht="238" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:31" ht="238">
       <c r="A96" s="4" t="s">
         <v>7</v>
       </c>
@@ -10779,7 +10779,7 @@
         <v>1020</v>
       </c>
     </row>
-    <row r="97" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:31" ht="255">
       <c r="A97" s="4" t="s">
         <v>7</v>
       </c>
@@ -10868,7 +10868,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="98" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:31" ht="17">
       <c r="A98" s="4" t="s">
         <v>7</v>
       </c>
@@ -10909,7 +10909,7 @@
       <c r="AD98" s="8"/>
       <c r="AE98" s="8"/>
     </row>
-    <row r="99" spans="1:31" ht="221" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:31" ht="221">
       <c r="A99" s="4" t="s">
         <v>7</v>
       </c>
@@ -11000,7 +11000,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="100" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:31" ht="17">
       <c r="A100" s="4" t="s">
         <v>7</v>
       </c>
@@ -11041,7 +11041,7 @@
       <c r="AD100" s="8"/>
       <c r="AE100" s="8"/>
     </row>
-    <row r="101" spans="1:31" ht="238" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:31" ht="238">
       <c r="A101" s="4" t="s">
         <v>7</v>
       </c>
@@ -11132,7 +11132,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="102" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:31" ht="17">
       <c r="A102" s="4" t="s">
         <v>7</v>
       </c>
@@ -11173,7 +11173,7 @@
       <c r="AD102" s="8"/>
       <c r="AE102" s="8"/>
     </row>
-    <row r="103" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:31" ht="255">
       <c r="A103" s="4" t="s">
         <v>10</v>
       </c>
@@ -11264,7 +11264,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="104" spans="1:31" ht="238" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:31" ht="238">
       <c r="A104" s="4" t="s">
         <v>7</v>
       </c>
@@ -11355,7 +11355,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="105" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:31" ht="17">
       <c r="A105" s="4" t="s">
         <v>7</v>
       </c>
@@ -11396,7 +11396,7 @@
       <c r="AD105" s="8"/>
       <c r="AE105" s="8"/>
     </row>
-    <row r="106" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:31" ht="17">
       <c r="A106" s="4" t="s">
         <v>7</v>
       </c>
@@ -11437,7 +11437,7 @@
       <c r="AD106" s="8"/>
       <c r="AE106" s="8"/>
     </row>
-    <row r="107" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:31" ht="289">
       <c r="A107" s="4" t="s">
         <v>7</v>
       </c>
@@ -11530,7 +11530,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="108" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:31" ht="17">
       <c r="A108" s="4" t="s">
         <v>7</v>
       </c>
@@ -11571,7 +11571,7 @@
       <c r="AD108" s="8"/>
       <c r="AE108" s="8"/>
     </row>
-    <row r="109" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:31" ht="255">
       <c r="A109" s="4" t="s">
         <v>7</v>
       </c>
@@ -11662,7 +11662,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="110" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:31" ht="17">
       <c r="A110" s="4" t="s">
         <v>7</v>
       </c>
@@ -11703,7 +11703,7 @@
       <c r="AD110" s="8"/>
       <c r="AE110" s="8"/>
     </row>
-    <row r="111" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:31" ht="289">
       <c r="A111" s="4" t="s">
         <v>7</v>
       </c>
@@ -11796,7 +11796,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="112" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:31" ht="17">
       <c r="A112" s="4" t="s">
         <v>7</v>
       </c>
@@ -11837,7 +11837,7 @@
       <c r="AD112" s="16"/>
       <c r="AE112" s="17"/>
     </row>
-    <row r="113" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:31" ht="289">
       <c r="A113" s="4" t="s">
         <v>7</v>
       </c>
@@ -11928,7 +11928,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="114" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:31" ht="255">
       <c r="A114" s="4" t="s">
         <v>7</v>
       </c>
@@ -12021,7 +12021,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="115" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:31" ht="17">
       <c r="A115" s="4" t="s">
         <v>7</v>
       </c>
@@ -12062,7 +12062,7 @@
       <c r="AD115" s="8"/>
       <c r="AE115" s="8"/>
     </row>
-    <row r="116" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:31" ht="255">
       <c r="A116" s="4" t="s">
         <v>7</v>
       </c>
@@ -12153,7 +12153,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="117" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:31" ht="272">
       <c r="A117" s="4" t="s">
         <v>7</v>
       </c>
@@ -12246,7 +12246,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="118" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:31" ht="17">
       <c r="A118" s="4" t="s">
         <v>7</v>
       </c>
@@ -12287,7 +12287,7 @@
       <c r="AD118" s="8"/>
       <c r="AE118" s="8"/>
     </row>
-    <row r="119" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:31" ht="255">
       <c r="A119" s="4" t="s">
         <v>10</v>
       </c>
@@ -12380,7 +12380,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="120" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:31" ht="289">
       <c r="A120" s="4" t="s">
         <v>7</v>
       </c>
@@ -12471,7 +12471,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="121" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:31" ht="17">
       <c r="A121" s="4" t="s">
         <v>7</v>
       </c>
@@ -12512,7 +12512,7 @@
       <c r="AD121" s="8"/>
       <c r="AE121" s="8"/>
     </row>
-    <row r="122" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:31" ht="17">
       <c r="A122" s="4" t="s">
         <v>10</v>
       </c>
@@ -12553,7 +12553,7 @@
       <c r="AD122" s="8"/>
       <c r="AE122" s="8"/>
     </row>
-    <row r="123" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:31" ht="255">
       <c r="A123" s="4" t="s">
         <v>7</v>
       </c>
@@ -12646,7 +12646,7 @@
         <v>1019</v>
       </c>
     </row>
-    <row r="124" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:31" ht="17">
       <c r="A124" s="4" t="s">
         <v>7</v>
       </c>
@@ -12687,7 +12687,7 @@
       <c r="AD124" s="8"/>
       <c r="AE124" s="8"/>
     </row>
-    <row r="125" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:31" ht="272">
       <c r="A125" s="4" t="s">
         <v>7</v>
       </c>
@@ -12778,7 +12778,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="126" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:31" ht="17">
       <c r="A126" s="4" t="s">
         <v>7</v>
       </c>
@@ -12819,7 +12819,7 @@
       <c r="AD126" s="8"/>
       <c r="AE126" s="8"/>
     </row>
-    <row r="127" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:31" ht="255">
       <c r="A127" s="4" t="s">
         <v>7</v>
       </c>
@@ -12912,7 +12912,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="128" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:31" ht="17">
       <c r="A128" s="4" t="s">
         <v>7</v>
       </c>
@@ -12953,7 +12953,7 @@
       <c r="AD128" s="8"/>
       <c r="AE128" s="8"/>
     </row>
-    <row r="129" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:31" ht="272">
       <c r="A129" s="4" t="s">
         <v>7</v>
       </c>
@@ -13044,7 +13044,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="130" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:31" ht="272">
       <c r="A130" s="4" t="s">
         <v>7</v>
       </c>
@@ -13135,7 +13135,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="131" spans="1:31" ht="340" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:31" ht="340">
       <c r="A131" s="4" t="s">
         <v>7</v>
       </c>
@@ -13226,7 +13226,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="132" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:31" ht="255">
       <c r="A132" s="4" t="s">
         <v>7</v>
       </c>
@@ -13319,7 +13319,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="133" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:31" ht="17">
       <c r="A133" s="4" t="s">
         <v>7</v>
       </c>
@@ -13360,7 +13360,7 @@
       <c r="AD133" s="8"/>
       <c r="AE133" s="8"/>
     </row>
-    <row r="134" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:31" ht="17">
       <c r="A134" s="4" t="s">
         <v>7</v>
       </c>
@@ -13401,7 +13401,7 @@
       <c r="AD134" s="8"/>
       <c r="AE134" s="8"/>
     </row>
-    <row r="135" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:31" ht="272">
       <c r="A135" s="4" t="s">
         <v>7</v>
       </c>
@@ -13492,7 +13492,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="136" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:31" ht="17">
       <c r="A136" s="4" t="s">
         <v>7</v>
       </c>
@@ -13533,7 +13533,7 @@
       <c r="AD136" s="8"/>
       <c r="AE136" s="8"/>
     </row>
-    <row r="137" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:31" ht="17">
       <c r="A137" s="4" t="s">
         <v>7</v>
       </c>
@@ -13574,7 +13574,7 @@
       <c r="AD137" s="8"/>
       <c r="AE137" s="8"/>
     </row>
-    <row r="138" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:31" ht="17">
       <c r="A138" s="4" t="s">
         <v>7</v>
       </c>
@@ -13615,7 +13615,7 @@
       <c r="AD138" s="8"/>
       <c r="AE138" s="8"/>
     </row>
-    <row r="139" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:31" ht="255">
       <c r="A139" s="4" t="s">
         <v>7</v>
       </c>
@@ -13706,7 +13706,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="140" spans="1:31" ht="238" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:31" ht="238">
       <c r="A140" s="4" t="s">
         <v>10</v>
       </c>
@@ -13797,7 +13797,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="141" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:31" ht="255">
       <c r="A141" s="4" t="s">
         <v>7</v>
       </c>
@@ -13844,7 +13844,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="142" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:31" ht="272">
       <c r="A142" s="4" t="s">
         <v>10</v>
       </c>
@@ -13935,7 +13935,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="143" spans="1:31" ht="306" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:31" ht="306">
       <c r="A143" s="4" t="s">
         <v>10</v>
       </c>
@@ -14028,7 +14028,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="144" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:31" ht="17">
       <c r="A144" s="4" t="s">
         <v>7</v>
       </c>
@@ -14069,7 +14069,7 @@
       <c r="AD144" s="8"/>
       <c r="AE144" s="8"/>
     </row>
-    <row r="145" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:31" ht="272">
       <c r="A145" s="4" t="s">
         <v>7</v>
       </c>
@@ -14160,7 +14160,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="146" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:31" ht="272">
       <c r="A146" s="4" t="s">
         <v>7</v>
       </c>
@@ -14251,7 +14251,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="147" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:31" ht="255">
       <c r="A147" s="4" t="s">
         <v>7</v>
       </c>
@@ -14342,7 +14342,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="148" spans="1:31" ht="238" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:31" ht="238">
       <c r="A148" s="4" t="s">
         <v>10</v>
       </c>
@@ -14433,7 +14433,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="149" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:31" ht="17">
       <c r="A149" s="4" t="s">
         <v>7</v>
       </c>
@@ -14474,7 +14474,7 @@
       <c r="AD149" s="8"/>
       <c r="AE149" s="8"/>
     </row>
-    <row r="150" spans="1:31" ht="51" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:31" ht="51">
       <c r="A150" s="4" t="s">
         <v>7</v>
       </c>
@@ -14519,7 +14519,7 @@
       </c>
       <c r="AE150" s="8"/>
     </row>
-    <row r="151" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:31" ht="255">
       <c r="A151" s="4" t="s">
         <v>7</v>
       </c>
@@ -14610,7 +14610,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="152" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:31" ht="17">
       <c r="A152" s="4" t="s">
         <v>7</v>
       </c>
@@ -14651,7 +14651,7 @@
       <c r="AD152" s="8"/>
       <c r="AE152" s="8"/>
     </row>
-    <row r="153" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:31" ht="272">
       <c r="A153" s="4" t="s">
         <v>7</v>
       </c>
@@ -14744,7 +14744,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="154" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:31" ht="17">
       <c r="A154" s="4" t="s">
         <v>7</v>
       </c>
@@ -14785,7 +14785,7 @@
       <c r="AD154" s="8"/>
       <c r="AE154" s="8"/>
     </row>
-    <row r="155" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:31" ht="255">
       <c r="A155" s="4" t="s">
         <v>7</v>
       </c>
@@ -14878,7 +14878,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="156" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:31" ht="17">
       <c r="A156" s="4" t="s">
         <v>7</v>
       </c>
@@ -14919,7 +14919,7 @@
       <c r="AD156" s="8"/>
       <c r="AE156" s="8"/>
     </row>
-    <row r="157" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:31" ht="17">
       <c r="A157" s="4" t="s">
         <v>7</v>
       </c>
@@ -14960,7 +14960,7 @@
       <c r="AD157" s="16"/>
       <c r="AE157" s="17"/>
     </row>
-    <row r="158" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:31" ht="17">
       <c r="A158" s="4" t="s">
         <v>7</v>
       </c>
@@ -15001,7 +15001,7 @@
       <c r="AD158" s="16"/>
       <c r="AE158" s="17"/>
     </row>
-    <row r="159" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:31" ht="17">
       <c r="A159" s="4" t="s">
         <v>7</v>
       </c>
@@ -15042,7 +15042,7 @@
       <c r="AD159" s="8"/>
       <c r="AE159" s="8"/>
     </row>
-    <row r="160" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:31" ht="17">
       <c r="A160" s="4" t="s">
         <v>7</v>
       </c>
@@ -15083,7 +15083,7 @@
       <c r="AD160" s="8"/>
       <c r="AE160" s="8"/>
     </row>
-    <row r="161" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:31" ht="272">
       <c r="A161" s="4" t="s">
         <v>7</v>
       </c>
@@ -15174,7 +15174,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="162" spans="1:31" ht="323" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:31" ht="323">
       <c r="A162" s="4" t="s">
         <v>7</v>
       </c>
@@ -15267,7 +15267,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="163" spans="1:31" ht="238" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:31" ht="238">
       <c r="A163" s="4" t="s">
         <v>7</v>
       </c>
@@ -15358,7 +15358,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="164" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:31" ht="17">
       <c r="A164" s="4" t="s">
         <v>7</v>
       </c>
@@ -15399,7 +15399,7 @@
       <c r="AD164" s="8"/>
       <c r="AE164" s="8"/>
     </row>
-    <row r="165" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:31" ht="255">
       <c r="A165" s="4" t="s">
         <v>7</v>
       </c>
@@ -15492,7 +15492,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="166" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:31" ht="17">
       <c r="A166" s="4" t="s">
         <v>7</v>
       </c>
@@ -15533,7 +15533,7 @@
       <c r="AD166" s="8"/>
       <c r="AE166" s="8"/>
     </row>
-    <row r="167" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:31" ht="17">
       <c r="A167" s="4" t="s">
         <v>7</v>
       </c>
@@ -15574,7 +15574,7 @@
       <c r="AD167" s="8"/>
       <c r="AE167" s="8"/>
     </row>
-    <row r="168" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:31" ht="17">
       <c r="A168" s="4" t="s">
         <v>7</v>
       </c>
@@ -15615,7 +15615,7 @@
       <c r="AD168" s="8"/>
       <c r="AE168" s="8"/>
     </row>
-    <row r="169" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:31" ht="17">
       <c r="A169" s="4" t="s">
         <v>7</v>
       </c>
@@ -15656,7 +15656,7 @@
       <c r="AD169" s="8"/>
       <c r="AE169" s="8"/>
     </row>
-    <row r="170" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:31" ht="17">
       <c r="A170" s="4" t="s">
         <v>7</v>
       </c>
@@ -15697,7 +15697,7 @@
       <c r="AD170" s="8"/>
       <c r="AE170" s="8"/>
     </row>
-    <row r="171" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:31" ht="255">
       <c r="A171" s="4" t="s">
         <v>7</v>
       </c>
@@ -15788,7 +15788,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="172" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:31" ht="272">
       <c r="A172" s="4" t="s">
         <v>7</v>
       </c>
@@ -15881,7 +15881,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="173" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:31" ht="289">
       <c r="A173" s="4" t="s">
         <v>7</v>
       </c>
@@ -15974,7 +15974,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="174" spans="1:31" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:31" ht="409.6">
       <c r="A174" s="4" t="s">
         <v>7</v>
       </c>
@@ -16067,7 +16067,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="175" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:31" ht="289">
       <c r="A175" s="4" t="s">
         <v>10</v>
       </c>
@@ -16158,7 +16158,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="176" spans="1:31" ht="404" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:31" ht="404">
       <c r="A176" s="4" t="s">
         <v>7</v>
       </c>
@@ -16251,7 +16251,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="177" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:31" ht="17">
       <c r="A177" s="4" t="s">
         <v>7</v>
       </c>
@@ -16292,7 +16292,7 @@
       <c r="AD177" s="28"/>
       <c r="AE177" s="8"/>
     </row>
-    <row r="178" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:31" ht="17">
       <c r="A178" s="4" t="s">
         <v>7</v>
       </c>
@@ -16333,7 +16333,7 @@
       <c r="AD178" s="8"/>
       <c r="AE178" s="8"/>
     </row>
-    <row r="179" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:31" ht="255">
       <c r="A179" s="4" t="s">
         <v>7</v>
       </c>
@@ -16424,7 +16424,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="180" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:31" ht="17">
       <c r="A180" s="4" t="s">
         <v>7</v>
       </c>
@@ -16465,7 +16465,7 @@
       <c r="AD180" s="28"/>
       <c r="AE180" s="8"/>
     </row>
-    <row r="181" spans="1:31" ht="238" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:31" ht="238">
       <c r="A181" s="4" t="s">
         <v>7</v>
       </c>
@@ -16558,7 +16558,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="182" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:31" ht="17">
       <c r="A182" s="4" t="s">
         <v>7</v>
       </c>
@@ -16599,7 +16599,7 @@
       <c r="AD182" s="8"/>
       <c r="AE182" s="8"/>
     </row>
-    <row r="183" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:31" ht="255">
       <c r="A183" s="4" t="s">
         <v>7</v>
       </c>
@@ -16690,7 +16690,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="184" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:31" ht="17">
       <c r="A184" s="4" t="s">
         <v>7</v>
       </c>
@@ -16731,7 +16731,7 @@
       <c r="AD184" s="8"/>
       <c r="AE184" s="8"/>
     </row>
-    <row r="185" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:31" ht="272">
       <c r="A185" s="4" t="s">
         <v>7</v>
       </c>
@@ -16822,7 +16822,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="186" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:31" ht="17">
       <c r="A186" s="4" t="s">
         <v>7</v>
       </c>
@@ -16863,7 +16863,7 @@
       <c r="AD186" s="8"/>
       <c r="AE186" s="8"/>
     </row>
-    <row r="187" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:31" ht="289">
       <c r="A187" s="4" t="s">
         <v>7</v>
       </c>
@@ -16954,7 +16954,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="188" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:31" ht="17">
       <c r="A188" s="4" t="s">
         <v>7</v>
       </c>
@@ -16995,7 +16995,7 @@
       <c r="AD188" s="8"/>
       <c r="AE188" s="8"/>
     </row>
-    <row r="189" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:31" ht="255">
       <c r="A189" s="4" t="s">
         <v>10</v>
       </c>
@@ -17086,7 +17086,7 @@
         <v>766</v>
       </c>
     </row>
-    <row r="190" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:31" ht="17">
       <c r="A190" s="4" t="s">
         <v>7</v>
       </c>
@@ -17127,7 +17127,7 @@
       <c r="AD190" s="8"/>
       <c r="AE190" s="8"/>
     </row>
-    <row r="191" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:31" ht="17">
       <c r="A191" s="4" t="s">
         <v>7</v>
       </c>
@@ -17168,7 +17168,7 @@
       <c r="AD191" s="8"/>
       <c r="AE191" s="8"/>
     </row>
-    <row r="192" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:31" ht="289">
       <c r="A192" s="4" t="s">
         <v>7</v>
       </c>
@@ -17261,7 +17261,7 @@
         <v>768</v>
       </c>
     </row>
-    <row r="193" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:31" ht="289">
       <c r="A193" s="4" t="s">
         <v>7</v>
       </c>
@@ -17354,7 +17354,7 @@
         <v>770</v>
       </c>
     </row>
-    <row r="194" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:31" ht="17">
       <c r="A194" s="4" t="s">
         <v>7</v>
       </c>
@@ -17395,7 +17395,7 @@
       <c r="AD194" s="8"/>
       <c r="AE194" s="8"/>
     </row>
-    <row r="195" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:31" ht="17">
       <c r="A195" s="4" t="s">
         <v>7</v>
       </c>
@@ -17434,7 +17434,7 @@
       <c r="AD195" s="8"/>
       <c r="AE195" s="8"/>
     </row>
-    <row r="196" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:31" ht="272">
       <c r="A196" s="4" t="s">
         <v>10</v>
       </c>
@@ -17525,7 +17525,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="197" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:31" ht="255">
       <c r="A197" s="4" t="s">
         <v>7</v>
       </c>
@@ -17616,7 +17616,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="198" spans="1:31" ht="238" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:31" ht="238">
       <c r="A198" s="4" t="s">
         <v>7</v>
       </c>
@@ -17707,7 +17707,7 @@
         <v>774</v>
       </c>
     </row>
-    <row r="199" spans="1:31" ht="238" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:31" ht="238">
       <c r="A199" s="4" t="s">
         <v>7</v>
       </c>
@@ -17800,7 +17800,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="200" spans="1:31" ht="238" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:31" ht="238">
       <c r="A200" s="4" t="s">
         <v>7</v>
       </c>
@@ -17891,7 +17891,7 @@
         <v>1036</v>
       </c>
     </row>
-    <row r="201" spans="1:31" ht="238" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:31" ht="238">
       <c r="A201" s="4" t="s">
         <v>10</v>
       </c>
@@ -17984,7 +17984,7 @@
         <v>779</v>
       </c>
     </row>
-    <row r="202" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:31" ht="17">
       <c r="A202" s="4" t="s">
         <v>7</v>
       </c>
@@ -18027,7 +18027,7 @@
       <c r="AD202" s="28"/>
       <c r="AE202" s="8"/>
     </row>
-    <row r="203" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:31" ht="255">
       <c r="A203" s="4" t="s">
         <v>7</v>
       </c>
@@ -18118,7 +18118,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="204" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:31" ht="17">
       <c r="A204" s="4" t="s">
         <v>7</v>
       </c>
@@ -18161,7 +18161,7 @@
       <c r="AD204" s="28"/>
       <c r="AE204" s="17"/>
     </row>
-    <row r="205" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:31" ht="255">
       <c r="A205" s="4" t="s">
         <v>10</v>
       </c>
@@ -18252,7 +18252,7 @@
         <v>783</v>
       </c>
     </row>
-    <row r="206" spans="1:31" ht="306" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:31" ht="306">
       <c r="A206" s="4" t="s">
         <v>10</v>
       </c>
@@ -18343,7 +18343,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="207" spans="1:31" ht="306" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:31" ht="306">
       <c r="A207" s="4" t="s">
         <v>7</v>
       </c>
@@ -18434,7 +18434,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="208" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:31" ht="272">
       <c r="A208" s="4" t="s">
         <v>7</v>
       </c>
@@ -18525,7 +18525,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="209" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:31" ht="255">
       <c r="A209" s="4" t="s">
         <v>7</v>
       </c>
@@ -18618,7 +18618,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="210" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:31" ht="272">
       <c r="A210" s="4" t="s">
         <v>7</v>
       </c>
@@ -18709,7 +18709,7 @@
         <v>793</v>
       </c>
     </row>
-    <row r="211" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:31" ht="17">
       <c r="A211" s="4" t="s">
         <v>7</v>
       </c>
@@ -18750,7 +18750,7 @@
       <c r="AD211" s="8"/>
       <c r="AE211" s="8"/>
     </row>
-    <row r="212" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:31" ht="255">
       <c r="A212" s="4" t="s">
         <v>7</v>
       </c>
@@ -18841,7 +18841,7 @@
         <v>795</v>
       </c>
     </row>
-    <row r="213" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:31" ht="255">
       <c r="A213" s="4" t="s">
         <v>7</v>
       </c>
@@ -18934,7 +18934,7 @@
         <v>797</v>
       </c>
     </row>
-    <row r="214" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:31" ht="17">
       <c r="A214" s="4" t="s">
         <v>7</v>
       </c>
@@ -18977,7 +18977,7 @@
       <c r="AD214" s="28"/>
       <c r="AE214" s="8"/>
     </row>
-    <row r="215" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:31" ht="289">
       <c r="A215" s="4" t="s">
         <v>7</v>
       </c>
@@ -19070,7 +19070,7 @@
         <v>799</v>
       </c>
     </row>
-    <row r="216" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:31" ht="255">
       <c r="A216" s="4" t="s">
         <v>7</v>
       </c>
@@ -19161,7 +19161,7 @@
         <v>801</v>
       </c>
     </row>
-    <row r="217" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:31" ht="17">
       <c r="A217" s="4" t="s">
         <v>7</v>
       </c>
@@ -19202,7 +19202,7 @@
       <c r="AD217" s="8"/>
       <c r="AE217" s="8"/>
     </row>
-    <row r="218" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:31" ht="17">
       <c r="A218" s="4" t="s">
         <v>7</v>
       </c>
@@ -19243,7 +19243,7 @@
       <c r="AD218" s="8"/>
       <c r="AE218" s="8"/>
     </row>
-    <row r="219" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:31" ht="289">
       <c r="A219" s="4" t="s">
         <v>7</v>
       </c>
@@ -19334,7 +19334,7 @@
         <v>803</v>
       </c>
     </row>
-    <row r="220" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:31" ht="17">
       <c r="A220" s="4" t="s">
         <v>7</v>
       </c>
@@ -19375,7 +19375,7 @@
       <c r="AD220" s="8"/>
       <c r="AE220" s="8"/>
     </row>
-    <row r="221" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:31" ht="17">
       <c r="A221" s="4" t="s">
         <v>7</v>
       </c>
@@ -19416,7 +19416,7 @@
       <c r="AD221" s="8"/>
       <c r="AE221" s="8"/>
     </row>
-    <row r="222" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:31" ht="255">
       <c r="A222" s="4" t="s">
         <v>7</v>
       </c>
@@ -19507,7 +19507,7 @@
         <v>805</v>
       </c>
     </row>
-    <row r="223" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:31" ht="17">
       <c r="A223" s="4" t="s">
         <v>7</v>
       </c>
@@ -19548,7 +19548,7 @@
       <c r="AD223" s="8"/>
       <c r="AE223" s="8"/>
     </row>
-    <row r="224" spans="1:31" ht="306" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:31" ht="306">
       <c r="A224" s="4" t="s">
         <v>7</v>
       </c>
@@ -19641,7 +19641,7 @@
         <v>807</v>
       </c>
     </row>
-    <row r="225" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:31" ht="289">
       <c r="A225" s="4" t="s">
         <v>10</v>
       </c>
@@ -19732,7 +19732,7 @@
         <v>811</v>
       </c>
     </row>
-    <row r="226" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:31" ht="17">
       <c r="A226" s="4" t="s">
         <v>7</v>
       </c>
@@ -19773,7 +19773,7 @@
       <c r="AD226" s="8"/>
       <c r="AE226" s="8"/>
     </row>
-    <row r="227" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:31" ht="17">
       <c r="A227" s="4" t="s">
         <v>7</v>
       </c>
@@ -19814,7 +19814,7 @@
       <c r="AD227" s="28"/>
       <c r="AE227" s="8"/>
     </row>
-    <row r="228" spans="1:31" ht="204" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:31" ht="204">
       <c r="A228" s="4" t="s">
         <v>10</v>
       </c>
@@ -19905,7 +19905,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="229" spans="1:31" ht="323" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:31" ht="323">
       <c r="A229" s="4" t="s">
         <v>7</v>
       </c>
@@ -19996,7 +19996,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="230" spans="1:31" ht="238" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:31" ht="238">
       <c r="A230" s="4" t="s">
         <v>7</v>
       </c>
@@ -20089,7 +20089,7 @@
         <v>813</v>
       </c>
     </row>
-    <row r="231" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:31" ht="255">
       <c r="A231" s="4" t="s">
         <v>7</v>
       </c>
@@ -20180,7 +20180,7 @@
         <v>815</v>
       </c>
     </row>
-    <row r="232" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:31" ht="17">
       <c r="A232" s="4" t="s">
         <v>7</v>
       </c>
@@ -20221,7 +20221,7 @@
       <c r="AD232" s="8"/>
       <c r="AE232" s="8"/>
     </row>
-    <row r="233" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:31" ht="17">
       <c r="A233" s="4" t="s">
         <v>7</v>
       </c>
@@ -20262,7 +20262,7 @@
       <c r="AD233" s="8"/>
       <c r="AE233" s="8"/>
     </row>
-    <row r="234" spans="1:31" ht="238" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:31" ht="238">
       <c r="A234" s="4" t="s">
         <v>7</v>
       </c>
@@ -20355,7 +20355,7 @@
         <v>817</v>
       </c>
     </row>
-    <row r="235" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:31" ht="289">
       <c r="A235" s="4" t="s">
         <v>7</v>
       </c>
@@ -20446,7 +20446,7 @@
         <v>819</v>
       </c>
     </row>
-    <row r="236" spans="1:31" ht="221" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:31" ht="221">
       <c r="A236" s="4" t="s">
         <v>7</v>
       </c>
@@ -20537,7 +20537,7 @@
         <v>943</v>
       </c>
     </row>
-    <row r="237" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:31" ht="289">
       <c r="A237" s="4" t="s">
         <v>7</v>
       </c>
@@ -20628,7 +20628,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="238" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:31" ht="255">
       <c r="A238" s="4" t="s">
         <v>7</v>
       </c>
@@ -20719,7 +20719,7 @@
         <v>824</v>
       </c>
     </row>
-    <row r="239" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:31" ht="17">
       <c r="A239" s="4" t="s">
         <v>7</v>
       </c>
@@ -20760,7 +20760,7 @@
       <c r="AD239" s="8"/>
       <c r="AE239" s="8"/>
     </row>
-    <row r="240" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:31" ht="17">
       <c r="A240" s="4" t="s">
         <v>7</v>
       </c>
@@ -20801,7 +20801,7 @@
       <c r="AD240" s="8"/>
       <c r="AE240" s="8"/>
     </row>
-    <row r="241" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:31" ht="17">
       <c r="A241" s="4" t="s">
         <v>7</v>
       </c>
@@ -20842,7 +20842,7 @@
       <c r="AD241" s="8"/>
       <c r="AE241" s="8"/>
     </row>
-    <row r="242" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:31" ht="255">
       <c r="A242" s="4" t="s">
         <v>7</v>
       </c>
@@ -20933,7 +20933,7 @@
         <v>829</v>
       </c>
     </row>
-    <row r="243" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:31" ht="17">
       <c r="A243" s="4" t="s">
         <v>7</v>
       </c>
@@ -20974,7 +20974,7 @@
       <c r="AD243" s="16"/>
       <c r="AE243" s="17"/>
     </row>
-    <row r="244" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:31" ht="17">
       <c r="A244" s="4" t="s">
         <v>7</v>
       </c>
@@ -21015,7 +21015,7 @@
       <c r="AD244" s="28"/>
       <c r="AE244" s="8"/>
     </row>
-    <row r="245" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:31" ht="255">
       <c r="A245" s="4" t="s">
         <v>7</v>
       </c>
@@ -21106,7 +21106,7 @@
         <v>831</v>
       </c>
     </row>
-    <row r="246" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:31" ht="17">
       <c r="A246" s="4" t="s">
         <v>7</v>
       </c>
@@ -21147,7 +21147,7 @@
       <c r="AD246" s="8"/>
       <c r="AE246" s="8"/>
     </row>
-    <row r="247" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:31" ht="17">
       <c r="A247" s="4" t="s">
         <v>7</v>
       </c>
@@ -21188,7 +21188,7 @@
       <c r="AD247" s="28"/>
       <c r="AE247" s="8"/>
     </row>
-    <row r="248" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:31" ht="272">
       <c r="A248" s="4" t="s">
         <v>7</v>
       </c>
@@ -21279,7 +21279,7 @@
         <v>962</v>
       </c>
     </row>
-    <row r="249" spans="1:31" ht="356" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:31" ht="356">
       <c r="A249" s="4" t="s">
         <v>7</v>
       </c>
@@ -21370,7 +21370,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="250" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:31" ht="272">
       <c r="A250" s="4" t="s">
         <v>7</v>
       </c>
@@ -21463,7 +21463,7 @@
         <v>963</v>
       </c>
     </row>
-    <row r="251" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:31" ht="17">
       <c r="A251" s="4" t="s">
         <v>7</v>
       </c>
@@ -21504,7 +21504,7 @@
       <c r="AD251" s="8"/>
       <c r="AE251" s="8"/>
     </row>
-    <row r="252" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:31" ht="17">
       <c r="A252" s="4" t="s">
         <v>7</v>
       </c>
@@ -21545,7 +21545,7 @@
       <c r="AD252" s="28"/>
       <c r="AE252" s="8"/>
     </row>
-    <row r="253" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:31" ht="17">
       <c r="A253" s="4" t="s">
         <v>7</v>
       </c>
@@ -21586,7 +21586,7 @@
       <c r="AD253" s="8"/>
       <c r="AE253" s="8"/>
     </row>
-    <row r="254" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:31" ht="17">
       <c r="A254" s="4" t="s">
         <v>7</v>
       </c>
@@ -21627,7 +21627,7 @@
       <c r="AD254" s="8"/>
       <c r="AE254" s="8"/>
     </row>
-    <row r="255" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:31" ht="17">
       <c r="A255" s="4" t="s">
         <v>7</v>
       </c>
@@ -21670,7 +21670,7 @@
       <c r="AD255" s="28"/>
       <c r="AE255" s="8"/>
     </row>
-    <row r="256" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:31" ht="17">
       <c r="A256" s="4" t="s">
         <v>7</v>
       </c>
@@ -21711,7 +21711,7 @@
       <c r="AD256" s="8"/>
       <c r="AE256" s="8"/>
     </row>
-    <row r="257" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:31" ht="17">
       <c r="A257" s="4" t="s">
         <v>7</v>
       </c>
@@ -21752,7 +21752,7 @@
       <c r="AD257" s="8"/>
       <c r="AE257" s="8"/>
     </row>
-    <row r="258" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:31" ht="289">
       <c r="A258" s="4" t="s">
         <v>7</v>
       </c>
@@ -21843,7 +21843,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="259" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:31" ht="17">
       <c r="A259" s="4" t="s">
         <v>7</v>
       </c>
@@ -21884,7 +21884,7 @@
       <c r="AD259" s="8"/>
       <c r="AE259" s="8"/>
     </row>
-    <row r="260" spans="1:31" ht="238" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:31" ht="238">
       <c r="A260" s="4" t="s">
         <v>7</v>
       </c>
@@ -21975,7 +21975,7 @@
         <v>828</v>
       </c>
     </row>
-    <row r="261" spans="1:31" ht="289" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:31" ht="289">
       <c r="A261" s="4" t="s">
         <v>7</v>
       </c>
@@ -22066,7 +22066,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="262" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:31" ht="17">
       <c r="A262" s="4" t="s">
         <v>7</v>
       </c>
@@ -22107,7 +22107,7 @@
       <c r="AD262" s="8"/>
       <c r="AE262" s="8"/>
     </row>
-    <row r="263" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:31" ht="17">
       <c r="A263" s="4" t="s">
         <v>7</v>
       </c>
@@ -22148,7 +22148,7 @@
       <c r="AD263" s="8"/>
       <c r="AE263" s="8"/>
     </row>
-    <row r="264" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:31" ht="17">
       <c r="A264" s="4" t="s">
         <v>7</v>
       </c>
@@ -22189,7 +22189,7 @@
       <c r="AD264" s="8"/>
       <c r="AE264" s="8"/>
     </row>
-    <row r="265" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:31" ht="17">
       <c r="A265" s="4" t="s">
         <v>7</v>
       </c>
@@ -22232,7 +22232,7 @@
       <c r="AD265" s="8"/>
       <c r="AE265" s="8"/>
     </row>
-    <row r="266" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:31" ht="255">
       <c r="A266" s="4" t="s">
         <v>10</v>
       </c>
@@ -22323,7 +22323,7 @@
         <v>965</v>
       </c>
     </row>
-    <row r="267" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:31" ht="272">
       <c r="A267" s="4" t="s">
         <v>10</v>
       </c>
@@ -22414,7 +22414,7 @@
         <v>966</v>
       </c>
     </row>
-    <row r="268" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:31" ht="17">
       <c r="A268" s="4" t="s">
         <v>7</v>
       </c>
@@ -22455,7 +22455,7 @@
       <c r="AD268" s="8"/>
       <c r="AE268" s="8"/>
     </row>
-    <row r="269" spans="1:31" ht="221" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:31" ht="221">
       <c r="A269" s="4" t="s">
         <v>7</v>
       </c>
@@ -22500,7 +22500,7 @@
         <v>967</v>
       </c>
     </row>
-    <row r="270" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:31" ht="17">
       <c r="A270" s="4" t="s">
         <v>7</v>
       </c>
@@ -22541,7 +22541,7 @@
       <c r="AD270" s="28"/>
       <c r="AE270" s="8"/>
     </row>
-    <row r="271" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:31" ht="17">
       <c r="A271" s="4" t="s">
         <v>10</v>
       </c>
@@ -22582,7 +22582,7 @@
       <c r="AD271" s="8"/>
       <c r="AE271" s="8"/>
     </row>
-    <row r="272" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:31" ht="17">
       <c r="A272" s="4" t="s">
         <v>7</v>
       </c>
@@ -22623,7 +22623,7 @@
       <c r="AD272" s="8"/>
       <c r="AE272" s="8"/>
     </row>
-    <row r="273" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:31" ht="17">
       <c r="A273" s="4" t="s">
         <v>10</v>
       </c>
@@ -22664,7 +22664,7 @@
       <c r="AD273" s="8"/>
       <c r="AE273" s="8"/>
     </row>
-    <row r="274" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:31" ht="17">
       <c r="A274" s="4" t="s">
         <v>7</v>
       </c>
@@ -22705,7 +22705,7 @@
       <c r="AD274" s="8"/>
       <c r="AE274" s="8"/>
     </row>
-    <row r="275" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:31" ht="17">
       <c r="A275" s="4" t="s">
         <v>10</v>
       </c>
@@ -22746,7 +22746,7 @@
       <c r="AD275" s="8"/>
       <c r="AE275" s="8"/>
     </row>
-    <row r="276" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:31" ht="17">
       <c r="A276" s="4" t="s">
         <v>10</v>
       </c>
@@ -22787,7 +22787,7 @@
       <c r="AD276" s="8"/>
       <c r="AE276" s="8"/>
     </row>
-    <row r="277" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:31" ht="17">
       <c r="A277" s="4" t="s">
         <v>7</v>
       </c>
@@ -22828,7 +22828,7 @@
       <c r="AD277" s="8"/>
       <c r="AE277" s="8"/>
     </row>
-    <row r="278" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:31" ht="17">
       <c r="A278" s="4" t="s">
         <v>10</v>
       </c>
@@ -22869,7 +22869,7 @@
       <c r="AD278" s="8"/>
       <c r="AE278" s="8"/>
     </row>
-    <row r="279" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:31" ht="255">
       <c r="A279" s="4" t="s">
         <v>10</v>
       </c>
@@ -22960,7 +22960,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="280" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:31" ht="17">
       <c r="A280" s="4" t="s">
         <v>10</v>
       </c>
@@ -23001,7 +23001,7 @@
       <c r="AD280" s="8"/>
       <c r="AE280" s="8"/>
     </row>
-    <row r="281" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:31" ht="17">
       <c r="A281" s="4" t="s">
         <v>10</v>
       </c>
@@ -23042,7 +23042,7 @@
       <c r="AD281" s="8"/>
       <c r="AE281" s="8"/>
     </row>
-    <row r="282" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:31" ht="17">
       <c r="A282" s="4" t="s">
         <v>10</v>
       </c>
@@ -23083,7 +23083,7 @@
       <c r="AD282" s="8"/>
       <c r="AE282" s="8"/>
     </row>
-    <row r="283" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:31" ht="17">
       <c r="A283" s="4" t="s">
         <v>7</v>
       </c>
@@ -23124,7 +23124,7 @@
       <c r="AD283" s="8"/>
       <c r="AE283" s="8"/>
     </row>
-    <row r="284" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:31" ht="17">
       <c r="A284" s="4" t="s">
         <v>7</v>
       </c>
@@ -23165,7 +23165,7 @@
       <c r="AD284" s="8"/>
       <c r="AE284" s="8"/>
     </row>
-    <row r="285" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:31" ht="17">
       <c r="A285" s="4" t="s">
         <v>7</v>
       </c>
@@ -23206,7 +23206,7 @@
       <c r="AD285" s="8"/>
       <c r="AE285" s="8"/>
     </row>
-    <row r="286" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:31" ht="17">
       <c r="A286" s="4" t="s">
         <v>10</v>
       </c>
@@ -23247,7 +23247,7 @@
       <c r="AD286" s="8"/>
       <c r="AE286" s="8"/>
     </row>
-    <row r="287" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:31" ht="17">
       <c r="A287" s="4" t="s">
         <v>10</v>
       </c>
@@ -23288,7 +23288,7 @@
       <c r="AD287" s="8"/>
       <c r="AE287" s="8"/>
     </row>
-    <row r="288" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:31" ht="17">
       <c r="A288" s="4" t="s">
         <v>10</v>
       </c>
@@ -23329,7 +23329,7 @@
       <c r="AD288" s="8"/>
       <c r="AE288" s="8"/>
     </row>
-    <row r="289" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:31" ht="17">
       <c r="A289" s="4" t="s">
         <v>7</v>
       </c>
@@ -23370,7 +23370,7 @@
       <c r="AD289" s="16"/>
       <c r="AE289" s="17"/>
     </row>
-    <row r="290" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:31" ht="17">
       <c r="A290" s="4" t="s">
         <v>7</v>
       </c>
@@ -23411,7 +23411,7 @@
       <c r="AD290" s="16"/>
       <c r="AE290" s="17"/>
     </row>
-    <row r="291" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:31" ht="17">
       <c r="A291" s="4" t="s">
         <v>7</v>
       </c>
@@ -23452,7 +23452,7 @@
       <c r="AD291" s="8"/>
       <c r="AE291" s="8"/>
     </row>
-    <row r="292" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:31" ht="17">
       <c r="A292" s="4" t="s">
         <v>10</v>
       </c>
@@ -23493,7 +23493,7 @@
       <c r="AD292" s="8"/>
       <c r="AE292" s="8"/>
     </row>
-    <row r="293" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:31" ht="17">
       <c r="A293" s="4" t="s">
         <v>7</v>
       </c>
@@ -23534,7 +23534,7 @@
       <c r="AD293" s="8"/>
       <c r="AE293" s="8"/>
     </row>
-    <row r="294" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:31" ht="17">
       <c r="A294" s="4" t="s">
         <v>10</v>
       </c>
@@ -23575,7 +23575,7 @@
       <c r="AD294" s="8"/>
       <c r="AE294" s="8"/>
     </row>
-    <row r="295" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:31" ht="17">
       <c r="A295" s="4" t="s">
         <v>10</v>
       </c>
@@ -23616,7 +23616,7 @@
       <c r="AD295" s="8"/>
       <c r="AE295" s="8"/>
     </row>
-    <row r="296" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:31" ht="17">
       <c r="A296" s="4" t="s">
         <v>10</v>
       </c>
@@ -23657,7 +23657,7 @@
       <c r="AD296" s="8"/>
       <c r="AE296" s="8"/>
     </row>
-    <row r="297" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:31" ht="17">
       <c r="A297" s="4" t="s">
         <v>7</v>
       </c>
@@ -23698,7 +23698,7 @@
       <c r="AD297" s="8"/>
       <c r="AE297" s="8"/>
     </row>
-    <row r="298" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:31" ht="17">
       <c r="A298" s="4" t="s">
         <v>7</v>
       </c>
@@ -23739,7 +23739,7 @@
       <c r="AD298" s="8"/>
       <c r="AE298" s="8"/>
     </row>
-    <row r="299" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:31" ht="17">
       <c r="A299" s="4" t="s">
         <v>10</v>
       </c>
@@ -23780,7 +23780,7 @@
       <c r="AD299" s="8"/>
       <c r="AE299" s="8"/>
     </row>
-    <row r="300" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="300" spans="1:31" ht="17">
       <c r="A300" s="4" t="s">
         <v>10</v>
       </c>
@@ -23821,7 +23821,7 @@
       <c r="AD300" s="8"/>
       <c r="AE300" s="8"/>
     </row>
-    <row r="301" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="301" spans="1:31" ht="17">
       <c r="A301" s="4" t="s">
         <v>7</v>
       </c>
@@ -23862,7 +23862,7 @@
       <c r="AD301" s="8"/>
       <c r="AE301" s="8"/>
     </row>
-    <row r="302" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="302" spans="1:31" ht="17">
       <c r="A302" s="4" t="s">
         <v>7</v>
       </c>
@@ -23903,7 +23903,7 @@
       <c r="AD302" s="8"/>
       <c r="AE302" s="8"/>
     </row>
-    <row r="303" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="303" spans="1:31" ht="17">
       <c r="A303" s="4" t="s">
         <v>10</v>
       </c>
@@ -23944,7 +23944,7 @@
       <c r="AD303" s="8"/>
       <c r="AE303" s="8"/>
     </row>
-    <row r="304" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="304" spans="1:31" ht="17">
       <c r="A304" s="4" t="s">
         <v>10</v>
       </c>
@@ -23985,7 +23985,7 @@
       <c r="AD304" s="8"/>
       <c r="AE304" s="8"/>
     </row>
-    <row r="305" spans="1:31" ht="272" x14ac:dyDescent="0.2">
+    <row r="305" spans="1:31" ht="272">
       <c r="A305" s="4" t="s">
         <v>10</v>
       </c>
@@ -24070,7 +24070,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="306" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="306" spans="1:31" ht="17">
       <c r="A306" s="4" t="s">
         <v>10</v>
       </c>
@@ -24111,7 +24111,7 @@
       <c r="AD306" s="8"/>
       <c r="AE306" s="8"/>
     </row>
-    <row r="307" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:31" ht="17">
       <c r="A307" s="4" t="s">
         <v>7</v>
       </c>
@@ -24152,7 +24152,7 @@
       <c r="AD307" s="8"/>
       <c r="AE307" s="8"/>
     </row>
-    <row r="308" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="308" spans="1:31" ht="17">
       <c r="A308" s="4" t="s">
         <v>7</v>
       </c>
@@ -24193,7 +24193,7 @@
       <c r="AD308" s="8"/>
       <c r="AE308" s="8"/>
     </row>
-    <row r="309" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="309" spans="1:31" ht="17">
       <c r="A309" s="4" t="s">
         <v>7</v>
       </c>
@@ -24234,7 +24234,7 @@
       <c r="AD309" s="8"/>
       <c r="AE309" s="8"/>
     </row>
-    <row r="310" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="310" spans="1:31" ht="17">
       <c r="A310" s="4" t="s">
         <v>7</v>
       </c>
@@ -24275,7 +24275,7 @@
       <c r="AD310" s="8"/>
       <c r="AE310" s="8"/>
     </row>
-    <row r="311" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:31" ht="17">
       <c r="A311" s="4" t="s">
         <v>10</v>
       </c>
@@ -24316,7 +24316,7 @@
       <c r="AD311" s="8"/>
       <c r="AE311" s="8"/>
     </row>
-    <row r="312" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="312" spans="1:31" ht="17">
       <c r="A312" s="4" t="s">
         <v>10</v>
       </c>
@@ -24357,7 +24357,7 @@
       <c r="AD312" s="8"/>
       <c r="AE312" s="8"/>
     </row>
-    <row r="313" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="313" spans="1:31" ht="17">
       <c r="A313" s="4" t="s">
         <v>10</v>
       </c>
@@ -24398,7 +24398,7 @@
       <c r="AD313" s="8"/>
       <c r="AE313" s="8"/>
     </row>
-    <row r="314" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="314" spans="1:31" ht="17">
       <c r="A314" s="4" t="s">
         <v>7</v>
       </c>
@@ -24439,7 +24439,7 @@
       <c r="AD314" s="8"/>
       <c r="AE314" s="8"/>
     </row>
-    <row r="315" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="315" spans="1:31" ht="17">
       <c r="A315" s="4" t="s">
         <v>10</v>
       </c>
@@ -24480,7 +24480,7 @@
       <c r="AD315" s="8"/>
       <c r="AE315" s="8"/>
     </row>
-    <row r="316" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="316" spans="1:31" ht="17">
       <c r="A316" s="4" t="s">
         <v>10</v>
       </c>
@@ -24521,7 +24521,7 @@
       <c r="AD316" s="8"/>
       <c r="AE316" s="8"/>
     </row>
-    <row r="317" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="317" spans="1:31" ht="17">
       <c r="A317" s="4" t="s">
         <v>10</v>
       </c>
@@ -24562,7 +24562,7 @@
       <c r="AD317" s="8"/>
       <c r="AE317" s="8"/>
     </row>
-    <row r="318" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="318" spans="1:31" ht="17">
       <c r="A318" s="4" t="s">
         <v>10</v>
       </c>
@@ -24603,7 +24603,7 @@
       <c r="AD318" s="8"/>
       <c r="AE318" s="8"/>
     </row>
-    <row r="319" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="319" spans="1:31" ht="17">
       <c r="A319" s="4" t="s">
         <v>10</v>
       </c>
@@ -24644,7 +24644,7 @@
       <c r="AD319" s="8"/>
       <c r="AE319" s="8"/>
     </row>
-    <row r="320" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="320" spans="1:31" ht="17">
       <c r="A320" s="4" t="s">
         <v>10</v>
       </c>
@@ -24685,7 +24685,7 @@
       <c r="AD320" s="8"/>
       <c r="AE320" s="8"/>
     </row>
-    <row r="321" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="321" spans="1:31" ht="17">
       <c r="A321" s="4" t="s">
         <v>10</v>
       </c>
@@ -24726,7 +24726,7 @@
       <c r="AD321" s="8"/>
       <c r="AE321" s="8"/>
     </row>
-    <row r="322" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="322" spans="1:31" ht="17">
       <c r="A322" s="4" t="s">
         <v>10</v>
       </c>
@@ -24767,7 +24767,7 @@
       <c r="AD322" s="8"/>
       <c r="AE322" s="8"/>
     </row>
-    <row r="323" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="323" spans="1:31" ht="17">
       <c r="A323" s="4" t="s">
         <v>7</v>
       </c>
@@ -24808,7 +24808,7 @@
       <c r="AD323" s="8"/>
       <c r="AE323" s="8"/>
     </row>
-    <row r="324" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="324" spans="1:31" ht="17">
       <c r="A324" s="4" t="s">
         <v>10</v>
       </c>
@@ -24849,7 +24849,7 @@
       <c r="AD324" s="8"/>
       <c r="AE324" s="8"/>
     </row>
-    <row r="325" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="325" spans="1:31" ht="17">
       <c r="A325" s="4" t="s">
         <v>10</v>
       </c>
@@ -24890,7 +24890,7 @@
       <c r="AD325" s="8"/>
       <c r="AE325" s="8"/>
     </row>
-    <row r="326" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="326" spans="1:31" ht="17">
       <c r="A326" s="4" t="s">
         <v>10</v>
       </c>
@@ -24931,7 +24931,7 @@
       <c r="AD326" s="8"/>
       <c r="AE326" s="8"/>
     </row>
-    <row r="327" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="327" spans="1:31" ht="17">
       <c r="A327" s="4" t="s">
         <v>7</v>
       </c>
@@ -24972,7 +24972,7 @@
       <c r="AD327" s="8"/>
       <c r="AE327" s="8"/>
     </row>
-    <row r="328" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="328" spans="1:31" ht="17">
       <c r="A328" s="4" t="s">
         <v>10</v>
       </c>
@@ -25013,7 +25013,7 @@
       <c r="AD328" s="8"/>
       <c r="AE328" s="8"/>
     </row>
-    <row r="329" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="329" spans="1:31" ht="17">
       <c r="A329" s="4" t="s">
         <v>10</v>
       </c>
@@ -25054,7 +25054,7 @@
       <c r="AD329" s="8"/>
       <c r="AE329" s="8"/>
     </row>
-    <row r="330" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="330" spans="1:31" ht="17">
       <c r="A330" s="4" t="s">
         <v>10</v>
       </c>
@@ -25095,7 +25095,7 @@
       <c r="AD330" s="8"/>
       <c r="AE330" s="8"/>
     </row>
-    <row r="331" spans="1:31" ht="255" x14ac:dyDescent="0.2">
+    <row r="331" spans="1:31" ht="255">
       <c r="A331" s="4" t="s">
         <v>10</v>
       </c>
@@ -25186,7 +25186,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="332" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="332" spans="1:31" ht="17">
       <c r="A332" s="4" t="s">
         <v>10</v>
       </c>
@@ -25227,7 +25227,7 @@
       <c r="AD332" s="8"/>
       <c r="AE332" s="8"/>
     </row>
-    <row r="333" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="333" spans="1:31" ht="17">
       <c r="A333" s="4" t="s">
         <v>7</v>
       </c>
@@ -25268,7 +25268,7 @@
       <c r="AD333" s="8"/>
       <c r="AE333" s="8"/>
     </row>
-    <row r="334" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="334" spans="1:31" ht="17">
       <c r="A334" s="4" t="s">
         <v>10</v>
       </c>
@@ -25309,7 +25309,7 @@
       <c r="AD334" s="16"/>
       <c r="AE334" s="17"/>
     </row>
-    <row r="335" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="335" spans="1:31" ht="17">
       <c r="A335" s="4" t="s">
         <v>10</v>
       </c>
@@ -25350,7 +25350,7 @@
       <c r="AD335" s="16"/>
       <c r="AE335" s="17"/>
     </row>
-    <row r="336" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="336" spans="1:31" ht="17">
       <c r="A336" s="4" t="s">
         <v>7</v>
       </c>
@@ -25391,7 +25391,7 @@
       <c r="AD336" s="8"/>
       <c r="AE336" s="8"/>
     </row>
-    <row r="337" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="337" spans="1:31" ht="17">
       <c r="A337" s="4" t="s">
         <v>7</v>
       </c>
@@ -25432,7 +25432,7 @@
       <c r="AD337" s="8"/>
       <c r="AE337" s="8"/>
     </row>
-    <row r="338" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="338" spans="1:31" ht="17">
       <c r="A338" s="4" t="s">
         <v>7</v>
       </c>
@@ -25473,7 +25473,7 @@
       <c r="AD338" s="8"/>
       <c r="AE338" s="8"/>
     </row>
-    <row r="339" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="339" spans="1:31" ht="17">
       <c r="A339" s="4" t="s">
         <v>10</v>
       </c>
@@ -25514,7 +25514,7 @@
       <c r="AD339" s="8"/>
       <c r="AE339" s="8"/>
     </row>
-    <row r="340" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="340" spans="1:31" ht="17">
       <c r="A340" s="4" t="s">
         <v>10</v>
       </c>
@@ -25555,7 +25555,7 @@
       <c r="AD340" s="8"/>
       <c r="AE340" s="8"/>
     </row>
-    <row r="341" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="341" spans="1:31" ht="17">
       <c r="A341" s="4" t="s">
         <v>7</v>
       </c>
@@ -25596,7 +25596,7 @@
       <c r="AD341" s="8"/>
       <c r="AE341" s="8"/>
     </row>
-    <row r="342" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="342" spans="1:31" ht="17">
       <c r="A342" s="4" t="s">
         <v>10</v>
       </c>
@@ -25637,7 +25637,7 @@
       <c r="AD342" s="8"/>
       <c r="AE342" s="8"/>
     </row>
-    <row r="343" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="343" spans="1:31" ht="17">
       <c r="A343" s="4" t="s">
         <v>10</v>
       </c>
@@ -25678,7 +25678,7 @@
       <c r="AD343" s="8"/>
       <c r="AE343" s="8"/>
     </row>
-    <row r="344" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="344" spans="1:31" ht="17">
       <c r="A344" s="4" t="s">
         <v>16</v>
       </c>
@@ -25719,7 +25719,7 @@
       <c r="AD344" s="8"/>
       <c r="AE344" s="8"/>
     </row>
-    <row r="345" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="345" spans="1:31" ht="17">
       <c r="A345" s="4" t="s">
         <v>16</v>
       </c>
@@ -25760,7 +25760,7 @@
       <c r="AD345" s="8"/>
       <c r="AE345" s="8"/>
     </row>
-    <row r="346" spans="1:31" ht="17" x14ac:dyDescent="0.2">
+    <row r="346" spans="1:31" ht="17">
       <c r="A346" s="4" t="s">
         <v>16</v>
       </c>

</xml_diff>